<commit_message>
almanya sheet adi duzeltildi
</commit_message>
<xml_diff>
--- a/templates/taslak_de.xlsx
+++ b/templates/taslak_de.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hakan.sahin\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70DF8844-8B78-44EC-9D42-5BAFD950A668}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41D0BBFE-B609-4537-9FD8-6471131E6A29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="taslak_be" sheetId="1" r:id="rId1"/>
+    <sheet name="taslak_de" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>

</xml_diff>